<commit_message>
Added WVS Gpt 4.1 standard prompt results
</commit_message>
<xml_diff>
--- a/data/WVS_Wave7_multiple_questions_selected.xlsx
+++ b/data/WVS_Wave7_multiple_questions_selected.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adeng/Documents/py/MLLM-Joint-Publication/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\University Code\MLLM-Joint-Publication\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D22E0A6-505A-0341-A546-453E7E47C74C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE85843E-98FA-4E7E-B22D-630D28D3BE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="15720" xr2:uid="{5E5B915F-D64D-44ED-8197-0044F60AB7BA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5E5B915F-D64D-44ED-8197-0044F60AB7BA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>Code</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -87,9 +87,6 @@
   </si>
   <si>
     <t>Q108</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>Q130</t>
@@ -144,7 +141,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -547,15 +544,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA70B749-A964-4B75-8C56-97BF5276E868}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="65.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="56.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="58.1640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="38.83203125" customWidth="1"/>
+    <col min="2" max="2" width="65.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="56.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="58.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -567,12 +564,12 @@
       </c>
       <c r="D1" s="4"/>
     </row>
-    <row r="2" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="45">
       <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>6</v>
@@ -581,40 +578,40 @@
       <c r="E2" s="3"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="75">
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="75">
       <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="45">
       <c r="A5" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="75">
       <c r="A6" s="7" t="s">
         <v>12</v>
       </c>
@@ -625,75 +622,70 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="60">
       <c r="A7" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="75">
       <c r="A8" s="7" t="s">
         <v>15</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="60">
+      <c r="A9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="45">
+      <c r="A10" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="75">
+      <c r="A11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="48" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="48" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="64" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>16</v>
-      </c>
+    </row>
+    <row r="15" spans="1:6" s="2" customFormat="1">
+      <c r="C15" s="3"/>
       <c r="E15" s="3"/>
     </row>
-    <row r="19" spans="4:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="4:5">
       <c r="D19" s="4"/>
       <c r="E19" s="5"/>
     </row>
-    <row r="20" spans="4:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="4:5">
       <c r="D20" s="4"/>
       <c r="E20" s="5"/>
     </row>

</xml_diff>